<commit_message>
Update models and scalers for thesis comparison
</commit_message>
<xml_diff>
--- a/Predictions/compare_single_stride_k5_next_tick_4models.xlsx
+++ b/Predictions/compare_single_stride_k5_next_tick_4models.xlsx
@@ -542,22 +542,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17.02690696716309</v>
+        <v>32.90938568115234</v>
       </c>
       <c r="C5" t="n">
-        <v>17.29586601257324</v>
+        <v>19.03206634521484</v>
       </c>
       <c r="D5" t="n">
-        <v>3.038800716400146</v>
+        <v>2.808969736099243</v>
       </c>
       <c r="E5" t="n">
-        <v>14.30096340179443</v>
+        <v>14.78880023956299</v>
       </c>
       <c r="F5" t="n">
-        <v>15.06158828735352</v>
+        <v>25.50203323364258</v>
       </c>
       <c r="G5" t="n">
-        <v>12.53815650939941</v>
+        <v>14.77543830871582</v>
       </c>
     </row>
     <row r="6">
@@ -567,22 +567,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33.26190948486328</v>
+        <v>34.35921478271484</v>
       </c>
       <c r="C6" t="n">
-        <v>12.86273288726807</v>
+        <v>16.65359497070312</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.3863142430782318</v>
+        <v>0.4846718609333038</v>
       </c>
       <c r="E6" t="n">
-        <v>14.08655452728271</v>
+        <v>12.08931064605713</v>
       </c>
       <c r="F6" t="n">
-        <v>19.05702590942383</v>
+        <v>24.3360710144043</v>
       </c>
       <c r="G6" t="n">
-        <v>7.140910625457764</v>
+        <v>12.57291984558105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>